<commit_message>
feat: add data consistency validation columns to ExportDataCP
Adds VAL-* columns (O-Z) to the Contenido sheet validating PO-ESTADO
CONSTRUCCION values, Ejecutado field completeness, PO-CARS vs Ejecutado
status, and PO-FECHA CONSTRUIDA/PO-SEMANA PROYECTO/PO-CARS consistency
using the same week-number formula as cesel-CP-UpdateWeekly, gated by
the contractual anchor to match that addin's actual skip behavior.
Also auto-syncs the Metrado/Auditoria PivotTable row ranges on export
and includes the manually widened pivot source ranges in the template.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CkjC5tFuPFpkF7QwnvPPLq
</commit_message>
<xml_diff>
--- a/BimManagement/BimManagement/Commands/ExportDataCP/Resources/TemplateReport.xlsx
+++ b/BimManagement/BimManagement/Commands/ExportDataCP/Resources/TemplateReport.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Developer\Autodesk\Revit\cesel-audit-models\BimManagement\BimManagement\Commands\ExportDataCP\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB470366-B7AD-47FF-98A3-5F52C5DA3742}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{240258AE-C107-4014-A7E7-681043D06922}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" activeTab="2" xr2:uid="{874C10DA-F89B-40BA-9549-22AF3452981B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{874C10DA-F89B-40BA-9549-22AF3452981B}"/>
   </bookViews>
   <sheets>
     <sheet name="Portada" sheetId="3" r:id="rId1"/>
@@ -23,7 +23,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="11" r:id="rId5"/>
+    <pivotCache cacheId="0" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="34">
   <si>
     <t>PO-WBS</t>
   </si>
@@ -141,6 +141,12 @@
   </si>
   <si>
     <t>VAL-OBSERVACIONES</t>
+  </si>
+  <si>
+    <t>VAL-SEMANA PROYECTO OK</t>
+  </si>
+  <si>
+    <t>VAL-SEMANA PROYECTO ESPERADO</t>
   </si>
 </sst>
 </file>
@@ -297,6 +303,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -310,126 +317,11 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="44">
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="2" tint="-0.749992370372631"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="2" tint="-0.749992370372631"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
+  <dxfs count="22">
     <dxf>
       <font>
         <color theme="0"/>
@@ -616,7 +508,7 @@
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="James Cabrera" refreshedDate="46255.792014583334" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{BC367C6E-7549-4E78-BB79-C87467145BD3}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="A1:X154" sheet="Contenido"/>
+    <worksheetSource ref="A1:Z154" sheet="Contenido"/>
   </cacheSource>
   <cacheFields count="24">
     <cacheField name="MODELO" numFmtId="0">
@@ -750,7 +642,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3D825A54-A8BB-4FAF-AB2E-C2A8072605A1}" name="ResumenGeneral" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" gridDropZones="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3D825A54-A8BB-4FAF-AB2E-C2A8072605A1}" name="ResumenGeneral" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" gridDropZones="1" multipleFieldFilters="0">
   <location ref="A3:D5" firstHeaderRow="2" firstDataRow="2" firstDataCol="3" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="24">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -817,37 +709,37 @@
     <dataField name="Sum of METRADO" fld="13" baseField="5" baseItem="0"/>
   </dataFields>
   <formats count="11">
-    <format dxfId="32">
+    <format dxfId="10">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="31">
+    <format dxfId="9">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="30">
+    <format dxfId="8">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="29">
+    <format dxfId="7">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="28">
+    <format dxfId="6">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="27">
+    <format dxfId="5">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="26">
+    <format dxfId="4">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="25">
+    <format dxfId="3">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="24">
+    <format dxfId="2">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="23">
+    <format dxfId="1">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="22">
+    <format dxfId="0">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -864,7 +756,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B0682C6F-09EA-4DA6-B25F-634B3AEE4851}" name="ResumenGeneral" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" gridDropZones="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B0682C6F-09EA-4DA6-B25F-634B3AEE4851}" name="ResumenGeneral" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" gridDropZones="1" multipleFieldFilters="0">
   <location ref="A3:N5" firstHeaderRow="2" firstDataRow="2" firstDataCol="8" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="24">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -958,37 +850,37 @@
     <pageField fld="11" hier="-1"/>
   </pageFields>
   <formats count="11">
-    <format dxfId="43">
+    <format dxfId="21">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="42">
+    <format dxfId="20">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0"/>
     </format>
-    <format dxfId="41">
+    <format dxfId="19">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="40">
+    <format dxfId="18">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="39">
+    <format dxfId="17">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="38">
+    <format dxfId="16">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0"/>
     </format>
-    <format dxfId="37">
+    <format dxfId="15">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0"/>
     </format>
-    <format dxfId="36">
+    <format dxfId="14">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0"/>
     </format>
-    <format dxfId="35">
+    <format dxfId="13">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="34">
+    <format dxfId="12">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0"/>
     </format>
-    <format dxfId="33">
+    <format dxfId="11">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -1322,78 +1214,78 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B4B46FD-295C-451D-8D14-BB210228FBCA}">
   <dimension ref="B1:K8"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="12" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="2" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="17" t="s">
+    <row r="1" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-    </row>
-    <row r="3" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+    </row>
+    <row r="3" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="2:11" ht="54" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="16"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
+    <row r="4" spans="2:11" ht="54" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="17"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="17"/>
       <c r="G4" s="6"/>
       <c r="H4" s="6"/>
     </row>
-    <row r="5" spans="2:11" ht="54" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B5" s="16"/>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="16"/>
+    <row r="5" spans="2:11" ht="54" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
     </row>
-    <row r="6" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="7" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="2" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19"/>
-      <c r="I7" s="19"/>
-      <c r="J7" s="19"/>
-      <c r="K7" s="19"/>
-    </row>
-    <row r="8" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="F7" s="20"/>
+      <c r="G7" s="20"/>
+      <c r="H7" s="20"/>
+      <c r="I7" s="20"/>
+      <c r="J7" s="20"/>
+      <c r="K7" s="20"/>
+    </row>
+    <row r="8" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="4" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
-      <c r="E8" s="20">
+      <c r="E8" s="21">
         <v>1817</v>
       </c>
-      <c r="F8" s="20"/>
-      <c r="G8" s="20"/>
-      <c r="H8" s="20"/>
-      <c r="I8" s="20"/>
-      <c r="J8" s="20"/>
-      <c r="K8" s="20"/>
+      <c r="F8" s="21"/>
+      <c r="G8" s="21"/>
+      <c r="H8" s="21"/>
+      <c r="I8" s="21"/>
+      <c r="J8" s="21"/>
+      <c r="K8" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -1411,18 +1303,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97239E96-F503-4422-B8BD-85ABD18EEA06}">
   <dimension ref="A1:F12"/>
-  <sheetFormatPr defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="34.07421875" customWidth="1"/>
-    <col min="2" max="2" width="47.69140625" customWidth="1"/>
+    <col min="1" max="1" width="34.109375" customWidth="1"/>
+    <col min="2" max="2" width="47.6640625" customWidth="1"/>
     <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.921875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.4609375" style="11" customWidth="1"/>
-    <col min="6" max="6" width="14.84375" style="11" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.84375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.44140625" style="11" customWidth="1"/>
+    <col min="6" max="6" width="14.88671875" style="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="12" customFormat="1" ht="19.850000000000001" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:6" s="12" customFormat="1" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
         <v>7</v>
       </c>
@@ -1432,15 +1324,15 @@
       <c r="E1" s="13"/>
       <c r="F1" s="13"/>
     </row>
-    <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="21"/>
+      <c r="D3" s="16"/>
       <c r="E3"/>
       <c r="F3"/>
     </row>
-    <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>17</v>
       </c>
@@ -1456,7 +1348,7 @@
       <c r="E4"/>
       <c r="F4"/>
     </row>
-    <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -1470,31 +1362,31 @@
       <c r="E5"/>
       <c r="F5"/>
     </row>
-    <row r="6" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E6"/>
       <c r="F6"/>
     </row>
-    <row r="7" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E7"/>
       <c r="F7"/>
     </row>
-    <row r="8" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E8"/>
       <c r="F8"/>
     </row>
-    <row r="9" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E9"/>
       <c r="F9"/>
     </row>
-    <row r="10" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E10"/>
       <c r="F10"/>
     </row>
-    <row r="11" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E11"/>
       <c r="F11"/>
     </row>
-    <row r="12" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E12"/>
       <c r="F12"/>
     </row>
@@ -1506,19 +1398,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10113796-C2EA-47E7-BB29-C27DB851E2A1}">
   <dimension ref="A1:N12"/>
-  <sheetFormatPr defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.765625" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="19.07421875" customWidth="1"/>
-    <col min="4" max="4" width="21.69140625" customWidth="1"/>
-    <col min="5" max="5" width="24.4609375" style="11" customWidth="1"/>
-    <col min="6" max="6" width="27.69140625" style="11" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.765625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.69140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.109375" customWidth="1"/>
+    <col min="4" max="4" width="21.6640625" customWidth="1"/>
+    <col min="5" max="5" width="24.44140625" style="11" customWidth="1"/>
+    <col min="6" max="6" width="27.6640625" style="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="12" customFormat="1" ht="19.850000000000001" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:14" s="12" customFormat="1" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
         <v>7</v>
       </c>
@@ -1528,17 +1420,17 @@
       <c r="E1" s="13"/>
       <c r="F1" s="13"/>
     </row>
-    <row r="3" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E3"/>
       <c r="F3"/>
-      <c r="I3" s="21"/>
-      <c r="J3" s="21"/>
-      <c r="K3" s="21"/>
-      <c r="L3" s="21"/>
-      <c r="M3" s="21"/>
-      <c r="N3" s="21"/>
-    </row>
-    <row r="4" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="I3" s="16"/>
+      <c r="J3" s="16"/>
+      <c r="K3" s="16"/>
+      <c r="L3" s="16"/>
+      <c r="M3" s="16"/>
+      <c r="N3" s="16"/>
+    </row>
+    <row r="4" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>17</v>
       </c>
@@ -1564,7 +1456,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -1596,31 +1488,31 @@
       <c r="M5" s="11"/>
       <c r="N5" s="11"/>
     </row>
-    <row r="6" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E6"/>
       <c r="F6"/>
     </row>
-    <row r="7" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E7"/>
       <c r="F7"/>
     </row>
-    <row r="8" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E8"/>
       <c r="F8"/>
     </row>
-    <row r="9" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E9"/>
       <c r="F9"/>
     </row>
-    <row r="10" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E10"/>
       <c r="F10"/>
     </row>
-    <row r="11" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E11"/>
       <c r="F11"/>
     </row>
-    <row r="12" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E12"/>
       <c r="F12"/>
     </row>
@@ -1631,27 +1523,27 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AAE71C7-031F-4BBF-99DF-AB099BF7E53B}">
-  <dimension ref="A1:X1"/>
-  <sheetFormatPr defaultColWidth="8.84375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:Z1"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="15.4609375" style="7" customWidth="1"/>
-    <col min="2" max="2" width="7.84375" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.4609375" style="7" customWidth="1"/>
+    <col min="1" max="1" width="15.44140625" style="7" customWidth="1"/>
+    <col min="2" max="2" width="7.88671875" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.44140625" style="7" customWidth="1"/>
     <col min="4" max="4" width="15" style="7" customWidth="1"/>
-    <col min="5" max="5" width="11.4609375" style="7" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.84375" style="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.53515625" style="10" customWidth="1"/>
-    <col min="8" max="8" width="13.4609375" style="7" customWidth="1"/>
-    <col min="9" max="9" width="20.4609375" style="10" customWidth="1"/>
-    <col min="10" max="10" width="18.84375" style="9" customWidth="1"/>
-    <col min="11" max="11" width="18.84375" style="7" customWidth="1"/>
-    <col min="12" max="12" width="10.84375" style="7" customWidth="1"/>
-    <col min="13" max="14" width="13.765625" style="7" customWidth="1"/>
-    <col min="15" max="24" width="10.84375" style="7" customWidth="1"/>
-    <col min="25" max="16384" width="8.84375" style="7"/>
+    <col min="5" max="5" width="11.44140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.88671875" style="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.5546875" style="10" customWidth="1"/>
+    <col min="8" max="8" width="13.44140625" style="7" customWidth="1"/>
+    <col min="9" max="9" width="20.44140625" style="10" customWidth="1"/>
+    <col min="10" max="10" width="18.88671875" style="9" customWidth="1"/>
+    <col min="11" max="11" width="18.88671875" style="7" customWidth="1"/>
+    <col min="12" max="12" width="10.88671875" style="7" customWidth="1"/>
+    <col min="13" max="14" width="13.77734375" style="7" customWidth="1"/>
+    <col min="15" max="26" width="10.88671875" style="7" customWidth="1"/>
+    <col min="27" max="16384" width="8.88671875" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="15" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:26" s="15" customFormat="1" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="14" t="s">
         <v>17</v>
       </c>
@@ -1719,9 +1611,15 @@
         <v>29</v>
       </c>
       <c r="W1" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="X1" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y1" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="X1" s="14" t="s">
+      <c r="Z1" s="14" t="s">
         <v>31</v>
       </c>
     </row>

</xml_diff>